<commit_message>
starting with gene expression analyses
</commit_message>
<xml_diff>
--- a/Part3_PRS/PRS plan.xlsx
+++ b/Part3_PRS/PRS plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\EHI_laterality\Part3_PRS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CA281D-3788-4A82-8E5E-E2FD3C35F11B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A29C6FB-EE4A-4EF9-B344-B8B439786F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5430" yWindow="-13860" windowWidth="19425" windowHeight="10305" xr2:uid="{2E559D2D-4EE3-42F9-BAD7-5E19FA97EA67}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{2E559D2D-4EE3-42F9-BAD7-5E19FA97EA67}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="22">
   <si>
     <t>INES</t>
   </si>
@@ -92,18 +92,46 @@
     <t>SE</t>
   </si>
   <si>
-    <t>PRS r² (%)</t>
-  </si>
-  <si>
-    <t>Full r² (%)</t>
+    <t xml:space="preserve">Full r² </t>
+  </si>
+  <si>
+    <t>PRS r²</t>
+  </si>
+  <si>
+    <t>Only BD (265)</t>
+  </si>
+  <si>
+    <t>Base model accounts for Age, Sex, PC1 and PC2</t>
+  </si>
+  <si>
+    <t>Sanity check</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -131,8 +159,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,13 +500,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1D14117-6741-403F-BDE9-8E36E38C1DB4}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -490,16 +524,16 @@
         <v>16</v>
       </c>
       <c r="F1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" t="s">
         <v>17</v>
-      </c>
-      <c r="G1" t="s">
-        <v>18</v>
       </c>
       <c r="H1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -509,8 +543,26 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D2" s="3">
+        <v>0.56031699999999995</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.17098099999999999</v>
+      </c>
+      <c r="F2" s="3">
+        <v>4.6494010000000002E-2</v>
+      </c>
+      <c r="G2" s="3">
+        <v>5.7890440000000001E-2</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1.049E-3</v>
+      </c>
+      <c r="I2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -520,8 +572,26 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D3" s="3">
+        <v>-5.5117000000000003</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1.7190000000000001</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1.6034340000000001E-2</v>
+      </c>
+      <c r="G3" s="3">
+        <v>2.364229E-2</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1.56E-3</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -531,8 +601,23 @@
       <c r="C4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D4" s="3">
+        <v>1.0039999999999999E-3</v>
+      </c>
+      <c r="E4" s="3">
+        <v>8.3769999999999997E-2</v>
+      </c>
+      <c r="F4" s="3">
+        <v>2.8514179999999999E-7</v>
+      </c>
+      <c r="G4" s="3">
+        <v>8.4633070000000005E-2</v>
+      </c>
+      <c r="H4">
+        <v>0.99099999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -540,10 +625,25 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.97682999999999998</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1.0665</v>
+      </c>
+      <c r="F5" s="3">
+        <v>3.1661829999999999E-3</v>
+      </c>
+      <c r="G5" s="3">
+        <v>5.1635739999999998E-3</v>
+      </c>
+      <c r="H5">
+        <v>0.36499999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -553,8 +653,23 @@
       <c r="C6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D6" s="3">
+        <v>5.2579999999999997E-3</v>
+      </c>
+      <c r="E6" s="3">
+        <v>5.3930999999999996E-3</v>
+      </c>
+      <c r="F6" s="3">
+        <v>2.8024289999999999E-3</v>
+      </c>
+      <c r="G6" s="3">
+        <v>3.0606629999999999E-2</v>
+      </c>
+      <c r="H6">
+        <v>0.33460000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -564,8 +679,23 @@
       <c r="C7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D7" s="3">
+        <v>-1.1278900000000001</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.88278000000000001</v>
+      </c>
+      <c r="F7" s="3">
+        <v>5.5124909999999996E-3</v>
+      </c>
+      <c r="G7" s="3">
+        <v>2.0308039999999999E-2</v>
+      </c>
+      <c r="H7">
+        <v>0.2064</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -575,8 +705,23 @@
       <c r="C8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D8" s="3">
+        <v>0.1646</v>
+      </c>
+      <c r="E8" s="3">
+        <v>7.1680099999999997E-2</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1.6691959999999999E-2</v>
+      </c>
+      <c r="G8" s="3">
+        <v>2.376586E-2</v>
+      </c>
+      <c r="H8" s="2">
+        <v>2.35E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -586,8 +731,26 @@
       <c r="C9" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D9" s="3">
+        <v>0.61343499999999995</v>
+      </c>
+      <c r="E9" s="3">
+        <v>9.3723000000000001E-2</v>
+      </c>
+      <c r="F9" s="3">
+        <v>9.3108099999999999E-2</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0.17774090000000001</v>
+      </c>
+      <c r="H9" s="1">
+        <v>5.9399999999999997E-11</v>
+      </c>
+      <c r="I9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -597,8 +760,23 @@
       <c r="C10" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D10" s="3">
+        <v>1.156315</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1.18451</v>
+      </c>
+      <c r="F10" s="3">
+        <v>3.658541E-3</v>
+      </c>
+      <c r="G10" s="3">
+        <v>5.6555360000000001E-3</v>
+      </c>
+      <c r="H10">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -608,8 +786,23 @@
       <c r="C11" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D11" s="3">
+        <v>5.3210000000000002E-3</v>
+      </c>
+      <c r="E11" s="3">
+        <v>5.9456999999999999E-3</v>
+      </c>
+      <c r="F11" s="3">
+        <v>2.4046459999999999E-3</v>
+      </c>
+      <c r="G11" s="3">
+        <v>3.0208840000000001E-2</v>
+      </c>
+      <c r="H11">
+        <v>0.3715</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -619,8 +812,23 @@
       <c r="C12" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D12" s="3">
+        <v>-0.61109000000000002</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0.96955000000000002</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1.37133E-3</v>
+      </c>
+      <c r="G12" s="3">
+        <v>1.616689E-2</v>
+      </c>
+      <c r="H12">
+        <v>0.52900000000000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -630,8 +838,23 @@
       <c r="C13" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D13" s="3">
+        <v>2.7175000000000001E-2</v>
+      </c>
+      <c r="E13" s="3">
+        <v>7.8819E-2</v>
+      </c>
+      <c r="F13" s="3">
+        <v>3.893821E-4</v>
+      </c>
+      <c r="G13" s="3">
+        <v>7.4632880000000002E-3</v>
+      </c>
+      <c r="H13">
+        <v>0.73099999999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -641,8 +864,23 @@
       <c r="C14" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D14" s="3">
+        <v>-0.170236</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0.162688</v>
+      </c>
+      <c r="F14" s="3">
+        <v>4.6023510000000002E-3</v>
+      </c>
+      <c r="G14" s="3">
+        <v>1.5998789999999999E-2</v>
+      </c>
+      <c r="H14" s="3">
+        <v>0.295381</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -651,6 +889,78 @@
       </c>
       <c r="C15" t="s">
         <v>13</v>
+      </c>
+      <c r="D15" s="3">
+        <v>-0.50750099999999998</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.22896900000000001</v>
+      </c>
+      <c r="F15" s="3">
+        <v>3.4740960000000001E-2</v>
+      </c>
+      <c r="G15" s="3">
+        <v>4.5513829999999998E-2</v>
+      </c>
+      <c r="H15" s="4">
+        <v>2.6700000000000002E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1.5092000000000001</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1.7344999999999999</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1.2202319999999999E-3</v>
+      </c>
+      <c r="G16" s="3">
+        <v>8.8286830000000004E-3</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0.38500000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="3">
+        <v>4.8228</v>
+      </c>
+      <c r="E17" s="3">
+        <v>2.5874999999999999</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1.001294E-2</v>
+      </c>
+      <c r="G17" s="3">
+        <v>1.430521E-2</v>
+      </c>
+      <c r="H17" s="5">
+        <v>6.3200000000000006E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>